<commit_message>
Samarkand R12 estimate: aryk length 4.2 m with one bridge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMcGkENVAoRmK9vPt9xr7W
</commit_message>
<xml_diff>
--- a/samarkand/estimate/samarkand-estimate-R12.xlsx
+++ b/samarkand/estimate/samarkand-estimate-R12.xlsx
@@ -345,7 +345,7 @@
     <t xml:space="preserve">Готовый арабский шатёр + стандартный диван</t>
   </si>
   <si>
-    <t xml:space="preserve">Арык 0,3 × 5,75 м по оси хауза (майоликовые борта, рециркуляция от хауза) + 2 мостика из камня</t>
+    <t xml:space="preserve">Арык 0,3 × 4,2 м по оси хауза до «Бухарского купола» (майоликовые борта, рециркуляция от хауза) + мостик из камня</t>
   </si>
   <si>
     <t xml:space="preserve">«Бухарский купол»: ротонда Ø1,8 — подиум, решётчатый барабан Ø0,9 с подвесами, 4 витрины-короба, кольцевой навес Ø2,3, свет, касса</t>
@@ -3085,22 +3085,22 @@
         <v>1</v>
       </c>
       <c r="E64" s="13" t="n">
-        <v>32000000</v>
+        <v>27000000</v>
       </c>
       <c r="F64" s="13" t="n">
         <f aca="false">D64*E64</f>
-        <v>32000000</v>
+        <v>27000000</v>
       </c>
       <c r="G64" s="13" t="n">
         <f aca="false">F64/$H$2</f>
-        <v>1230.76923076923</v>
+        <v>1038.46153846154</v>
       </c>
       <c r="H64" s="11"/>
       <c r="I64" s="11"/>
       <c r="J64" s="13"/>
       <c r="K64" s="13" t="n">
         <f aca="false">F64</f>
-        <v>32000000</v>
+        <v>27000000</v>
       </c>
       <c r="L64" s="8"/>
     </row>
@@ -3427,18 +3427,18 @@
       <c r="E74" s="17"/>
       <c r="F74" s="18" t="n">
         <f aca="false">SUM(F59:F73)</f>
-        <v>1182000000</v>
+        <v>1177000000</v>
       </c>
       <c r="G74" s="18" t="n">
         <f aca="false">F74/$H$2</f>
-        <v>45461.5384615385</v>
+        <v>45269.2307692308</v>
       </c>
       <c r="H74" s="19"/>
       <c r="I74" s="19"/>
       <c r="J74" s="17"/>
       <c r="K74" s="18" t="n">
         <f aca="false">SUM(K59:K73)</f>
-        <v>957000000</v>
+        <v>952000000</v>
       </c>
       <c r="L74" s="8"/>
     </row>
@@ -3928,18 +3928,18 @@
       <c r="E94" s="8"/>
       <c r="F94" s="8" t="n">
         <f aca="false">F9+F33+F42+F56+F74+F80+F88+F92</f>
-        <v>4323858000</v>
+        <v>4318858000</v>
       </c>
       <c r="G94" s="8" t="n">
         <f aca="false">F94/$H$2</f>
-        <v>166302.230769231</v>
+        <v>166109.923076923</v>
       </c>
       <c r="H94" s="9"/>
       <c r="I94" s="9"/>
       <c r="J94" s="8"/>
       <c r="K94" s="8" t="n">
         <f aca="false">K9+K33+K42+K56+K74+K80+K88+K92</f>
-        <v>3586290000</v>
+        <v>3581290000</v>
       </c>
       <c r="L94" s="8"/>
     </row>
@@ -3951,18 +3951,18 @@
       <c r="E95" s="8"/>
       <c r="F95" s="8" t="n">
         <f aca="false">F94*0.1</f>
-        <v>432385800</v>
+        <v>431885800</v>
       </c>
       <c r="G95" s="8" t="n">
         <f aca="false">F95/$H$2</f>
-        <v>16630.2230769231</v>
+        <v>16610.9923076923</v>
       </c>
       <c r="H95" s="9"/>
       <c r="I95" s="9"/>
       <c r="J95" s="8"/>
       <c r="K95" s="8" t="n">
         <f aca="false">K94*0.1</f>
-        <v>358629000</v>
+        <v>358129000</v>
       </c>
       <c r="L95" s="8"/>
     </row>
@@ -3998,22 +3998,22 @@
       <c r="E97" s="24"/>
       <c r="F97" s="24" t="n">
         <f aca="false">SUM(F94:F96)</f>
-        <v>4801243800</v>
+        <v>4795743800</v>
       </c>
       <c r="G97" s="24" t="n">
         <f aca="false">F97/$H$2</f>
-        <v>184663.223076923</v>
+        <v>184451.684615385</v>
       </c>
       <c r="H97" s="22"/>
       <c r="I97" s="22"/>
       <c r="J97" s="24"/>
       <c r="K97" s="24" t="n">
         <f aca="false">SUM(K94:K96)</f>
-        <v>3989919000</v>
+        <v>3984419000</v>
       </c>
       <c r="L97" s="24" t="n">
         <f aca="false">K97/$H$2</f>
-        <v>153458.423076923</v>
+        <v>153246.884615385</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4053,7 +4053,7 @@
       <c r="E100" s="8"/>
       <c r="F100" s="8" t="n">
         <f aca="false">F97/446.5</f>
-        <v>10753065.6215006</v>
+        <v>10740747.5923852</v>
       </c>
       <c r="G100" s="8"/>
       <c r="H100" s="9"/>
@@ -4070,7 +4070,7 @@
       <c r="E101" s="8"/>
       <c r="F101" s="8" t="n">
         <f aca="false">F97/171</f>
-        <v>28077449.122807</v>
+        <v>28045285.380117</v>
       </c>
       <c r="G101" s="8"/>
       <c r="H101" s="9"/>

</xml_diff>